<commit_message>
bulk location update integration done
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/LocationUpdateExcel.xlsx
+++ b/Jobs/Tasks/FileProcess/LocationUpdateExcel.xlsx
@@ -32,18 +32,9 @@
     <t>AG001</t>
   </si>
   <si>
-    <t>Office</t>
-  </si>
-  <si>
-    <t>HO</t>
-  </si>
-  <si>
     <t>Agency</t>
   </si>
   <si>
-    <t xml:space="preserve">Retail Agency </t>
-  </si>
-  <si>
     <t>LocationType</t>
   </si>
   <si>
@@ -54,6 +45,15 @@
   </si>
   <si>
     <t>CurrentSubChannel</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>AH</t>
+  </si>
+  <si>
+    <t>Area Head</t>
   </si>
 </sst>
 </file>
@@ -395,16 +395,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -412,16 +412,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
       <c r="E2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>